<commit_message>
Add faculty email scraping Batch 5: Rutgers, Cornell (Tier 2 begins); CIA skipped
36 new faculty rows (Rutgers 8, Cornell 28), bringing the master workbook to
14 schools and 506 total rows. Cleveland Institute of Art checked and
skipped - all sampled profile pages use a contact form instead of a public
email, making it Tier 3 in practice despite the brief's Tier 2 classification.

Rutgers turned out to have direct emails (better than expected); Cornell
required a full profile click-through with bio-text fallback classification,
same pattern as Ohio State. Fixed a URL-encoded "Name <email>" mailto format
on Rutgers and flagged a shared department mailbox on Cornell as
department_general rather than a personal address.
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Faculty Scraping/master_faculty.xlsx
+++ b/Dezi Art Prize Faculty Scraping/master_faculty.xlsx
@@ -19,6 +19,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NID Ahmedabad" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jamia Millia Islamia" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UIC" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rutgers" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cornell" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Temple-Tyler'!$A$7:$I$58</definedName>
@@ -33,6 +35,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'NID Ahmedabad'!$A$7:$I$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Jamia Millia Islamia'!$A$7:$I$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'UIC'!$A$7:$I$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Rutgers'!$A$7:$I$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Cornell'!$A$7:$I$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -4492,6 +4496,1914 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Country: United States</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>City: New Brunswick, NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Source: Rutgers University, Mason Gross School of the Arts - Art &amp; Design department faculty/staff page. Emails ARE visible directly on the listing (better than the research brief's Tier 2 classification implied) - no profile click-through needed. Only faculty whose title text names a specific medium were kept (e.g. 'Associate Professor in Photography'); generic titles ('Professor') with no medium signal were left out rather than guessed, since this page has no separate discipline field. One email format quirk: a few hrefs are 'mailto:Name &lt;email&gt;' URL-encoded rather than a bare address - the actual address was extracted from either form.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://www.masongross.rutgers.edu/degrees-programs/art-design/faculty-staff/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>school_name</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>faculty_name</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>email_type</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>date_extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Rutgers University, Mason Gross School of the Arts</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Jacqueline Thaw</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Chair Associate Professor in Design</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Art &amp; Design</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>thaw@mgsa.rutgers.edu</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://www.masongross.rutgers.edu/degrees-programs/art-design/faculty-staff/</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Rutgers University, Mason Gross School of the Arts</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Atif Akin</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MFA in Design Director Professor</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Art &amp; Design</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>aakin@mgsa.rutgers.edu</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://www.masongross.rutgers.edu/degrees-programs/art-design/faculty-staff/</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Rutgers University, Mason Gross School of the Arts</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Miranda Lichtenstein</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Associate Professor in Photography</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Art &amp; Design</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>mlichtenstein@mgsa.rutgers.edu</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://www.masongross.rutgers.edu/degrees-programs/art-design/faculty-staff/</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Rutgers University, Mason Gross School of the Arts</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Barbara Madsen</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Director of the Rutgers Printmaking Collaborative Professor</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Art &amp; Design</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Fiber and Material Arts</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>bmadsen@mgsa.rutgers.edu</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://www.masongross.rutgers.edu/degrees-programs/art-design/faculty-staff/</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Rutgers University, Mason Gross School of the Arts</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Mark Armijo McKnight</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Expanded Photography</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Art &amp; Design</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>mark.mcknight@rutgers.edu</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://www.masongross.rutgers.edu/degrees-programs/art-design/faculty-staff/</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Rutgers University, Mason Gross School of the Arts</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Jeanine Oleson</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Associate Professor, Sculpture Graduate Director, Visual Arts</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Art &amp; Design</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>jeanine.oleson@rutgers.edu</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://www.masongross.rutgers.edu/degrees-programs/art-design/faculty-staff/</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Rutgers University, Mason Gross School of the Arts</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Rhys Bambrick</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Visual Arts Coordinator, Sculpture</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Art &amp; Design</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>rhys.bambrick@rutgers.edu</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://www.masongross.rutgers.edu/degrees-programs/art-design/faculty-staff/</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Rutgers University, Mason Gross School of the Arts</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Sean Zujkowski</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Photo Area Coordinator</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Art &amp; Design</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>sdz18@mgsa.rutgers.edu</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://www.masongross.rutgers.edu/degrees-programs/art-design/faculty-staff/</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A7:I15"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Country: United States</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>City: Ithaca, NY</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Source: Cornell University, Department of Art (AAP) - /art/art-people listing (41 entries, 5 duplicates from dual program listings, deduped to 36 unique profiles) with emails only on individual profile pages - required a click-through pass like Ohio State. Medium classified from title/role text first, falling back to each profile's bio paragraph when the role alone was generic (e.g. 'Professor'). 5 rows have email_type=department_general: several visiting/affiliated faculty list the shared imagetext@cornell.edu program mailbox as their own contact on their profile page, not a personal address - flagged rather than treated as equivalent to a direct personal email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://aap.cornell.edu/art/art-people (plus 36 individual /people/&lt;slug&gt;/ pages)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>school_name</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>faculty_name</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>email_type</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>date_extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Paul Ramírez Jonas</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Chair</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>par237@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/paul-ramirez-jonas/</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Keith Obadike</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Director of Undergraduate Studies</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Filmmaking</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>kao83@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/keith-obadike/</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Joanna Malinowska</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Director of Graduate Studies in Creative Visual Arts</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>jmm828@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/joanna-malinowska/</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Nicholas Muellner</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Codirector, M.F.A. in Image Text and ITI Press</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>nrm72@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/nicholas-muellner/</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Catherine Taylor</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Codirector, M.F.A. in Image Text and ITI Press</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Filmmaking</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>cct29@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/catherine-taylor/</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Lou Fuchs</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Sculpture Studio Technician</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>lff37@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/lou-fuchs/</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Jackie Riccio</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Print Media, Drawing, and Painting Studio Technician</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>jr2452@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/jackie-riccio/</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Jennifer Gioffre Todd</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Director of Material Practice</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>jmg393@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/jennifer-gioffre-todd/</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Michael Ashkin</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>ma352@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/michael-ashkin/</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Oscar Rene Cornejo</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Assistant Professor</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>orc7@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/oscar-rene-cornejo/</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Jen de los Reyes</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Fiber and Material Arts</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>jd2276@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/jen-de-los-reyes/</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Leeza Meksin</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Assistant Professor</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>evm28@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/leeza-meksin/</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Elisabeth Meyer</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>ehm2@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/elisabeth-meyer/</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Carl Ostendarp</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>cao24@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/carl-ostendarp/</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Maria Park</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>myp4@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/maria-park/</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Leslie Brack</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>lb624@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/leslie-brack/</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Carla Liesching</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>cel242@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/carla-liesching/</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Matt Bollinger</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Visiting Critic</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>mlb522@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/matt-bollinger/</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Mark Anthony Brown Jr.</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Strauch Early Career Fellow</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>mab692@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/mark-anthony-brown-jr/</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Matthew Connors</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Visiting Critic (summer 2026)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>imagetext@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>department_general</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/matthew-connors/</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Claire Donato</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Visiting Critic (summer and fall 2026)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Filmmaking</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>imagetext@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>department_general</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/claire-donato/</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Whitney Hubbs</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Visiting Critic (summer and fall 2026)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>weh62@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/whitney-hubbs/</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Kyle Bellucci Johanson</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Visiting Critic</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>kj368@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/kyle-bellucci-johanson/</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Ben Rivers</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Visiting Critic (summer 2026)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Filmmaking</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>imagetext@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>department_general</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/ben-rivers/</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Keisha Scarville</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Visiting Critic (fall 2026)</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>imagetext@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>department_general</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/keisha-scarville/</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Paulina Velázquez Solís</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Visiting Critic</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>pv233@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/paulina-velazquez-solis/</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Carla Williams</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Visiting Critic (summer 2026)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>imagetext@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>department_general</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/carla-williams/</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Carmen Winant</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Visiting Critic (summer 2026)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>cw297@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/carmen-winant/</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A7:I35"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update master_faculty.xlsx with Batch 5 (Rutgers, Cornell) - 506 total rows
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Faculty Scraping/master_faculty.xlsx
+++ b/Dezi Art Prize Faculty Scraping/master_faculty.xlsx
@@ -19,6 +19,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NID Ahmedabad" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jamia Millia Islamia" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UIC" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rutgers" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cornell" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Temple-Tyler'!$A$7:$I$58</definedName>
@@ -33,6 +35,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'NID Ahmedabad'!$A$7:$I$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Jamia Millia Islamia'!$A$7:$I$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'UIC'!$A$7:$I$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Rutgers'!$A$7:$I$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Cornell'!$A$7:$I$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -4492,6 +4496,1914 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Country: United States</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>City: New Brunswick, NJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Source: Rutgers University, Mason Gross School of the Arts - Art &amp; Design department faculty/staff page. Emails ARE visible directly on the listing (better than the research brief's Tier 2 classification implied) - no profile click-through needed. Only faculty whose title text names a specific medium were kept (e.g. 'Associate Professor in Photography'); generic titles ('Professor') with no medium signal were left out rather than guessed, since this page has no separate discipline field. One email format quirk: a few hrefs are 'mailto:Name &lt;email&gt;' URL-encoded rather than a bare address - the actual address was extracted from either form.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://www.masongross.rutgers.edu/degrees-programs/art-design/faculty-staff/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>school_name</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>faculty_name</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>email_type</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>date_extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Rutgers University, Mason Gross School of the Arts</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Jacqueline Thaw</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Chair Associate Professor in Design</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Art &amp; Design</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>thaw@mgsa.rutgers.edu</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://www.masongross.rutgers.edu/degrees-programs/art-design/faculty-staff/</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Rutgers University, Mason Gross School of the Arts</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Atif Akin</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MFA in Design Director Professor</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Art &amp; Design</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>aakin@mgsa.rutgers.edu</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://www.masongross.rutgers.edu/degrees-programs/art-design/faculty-staff/</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Rutgers University, Mason Gross School of the Arts</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Miranda Lichtenstein</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Associate Professor in Photography</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Art &amp; Design</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>mlichtenstein@mgsa.rutgers.edu</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://www.masongross.rutgers.edu/degrees-programs/art-design/faculty-staff/</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Rutgers University, Mason Gross School of the Arts</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Barbara Madsen</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Director of the Rutgers Printmaking Collaborative Professor</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Art &amp; Design</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Fiber and Material Arts</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>bmadsen@mgsa.rutgers.edu</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://www.masongross.rutgers.edu/degrees-programs/art-design/faculty-staff/</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Rutgers University, Mason Gross School of the Arts</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Mark Armijo McKnight</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Expanded Photography</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Art &amp; Design</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>mark.mcknight@rutgers.edu</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://www.masongross.rutgers.edu/degrees-programs/art-design/faculty-staff/</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Rutgers University, Mason Gross School of the Arts</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Jeanine Oleson</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Associate Professor, Sculpture Graduate Director, Visual Arts</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Art &amp; Design</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>jeanine.oleson@rutgers.edu</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://www.masongross.rutgers.edu/degrees-programs/art-design/faculty-staff/</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Rutgers University, Mason Gross School of the Arts</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Rhys Bambrick</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Visual Arts Coordinator, Sculpture</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Art &amp; Design</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>rhys.bambrick@rutgers.edu</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://www.masongross.rutgers.edu/degrees-programs/art-design/faculty-staff/</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Rutgers University, Mason Gross School of the Arts</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Sean Zujkowski</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Photo Area Coordinator</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Art &amp; Design</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>sdz18@mgsa.rutgers.edu</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://www.masongross.rutgers.edu/degrees-programs/art-design/faculty-staff/</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A7:I15"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Country: United States</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>City: Ithaca, NY</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Source: Cornell University, Department of Art (AAP) - /art/art-people listing (41 entries, 5 duplicates from dual program listings, deduped to 36 unique profiles) with emails only on individual profile pages - required a click-through pass like Ohio State. Medium classified from title/role text first, falling back to each profile's bio paragraph when the role alone was generic (e.g. 'Professor'). 5 rows have email_type=department_general: several visiting/affiliated faculty list the shared imagetext@cornell.edu program mailbox as their own contact on their profile page, not a personal address - flagged rather than treated as equivalent to a direct personal email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://aap.cornell.edu/art/art-people (plus 36 individual /people/&lt;slug&gt;/ pages)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>school_name</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>faculty_name</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>email_type</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>date_extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Paul Ramírez Jonas</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Chair</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>par237@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/paul-ramirez-jonas/</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Keith Obadike</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Director of Undergraduate Studies</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Filmmaking</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>kao83@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/keith-obadike/</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Joanna Malinowska</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Director of Graduate Studies in Creative Visual Arts</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>jmm828@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/joanna-malinowska/</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Nicholas Muellner</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Codirector, M.F.A. in Image Text and ITI Press</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>nrm72@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/nicholas-muellner/</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Catherine Taylor</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Codirector, M.F.A. in Image Text and ITI Press</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Filmmaking</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>cct29@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/catherine-taylor/</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Lou Fuchs</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Sculpture Studio Technician</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>lff37@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/lou-fuchs/</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Jackie Riccio</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Print Media, Drawing, and Painting Studio Technician</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>jr2452@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/jackie-riccio/</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Jennifer Gioffre Todd</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Director of Material Practice</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>jmg393@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/jennifer-gioffre-todd/</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Michael Ashkin</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Professor</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>ma352@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/michael-ashkin/</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Oscar Rene Cornejo</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Assistant Professor</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>orc7@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/oscar-rene-cornejo/</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Jen de los Reyes</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Fiber and Material Arts</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>jd2276@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/jen-de-los-reyes/</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Leeza Meksin</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Assistant Professor</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>evm28@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/leeza-meksin/</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Elisabeth Meyer</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>ehm2@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/elisabeth-meyer/</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Carl Ostendarp</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>cao24@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/carl-ostendarp/</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Maria Park</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Associate Professor</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>myp4@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/maria-park/</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Leslie Brack</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>lb624@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/leslie-brack/</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Carla Liesching</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Lecturer</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>cel242@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/carla-liesching/</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Matt Bollinger</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Visiting Critic</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>mlb522@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/matt-bollinger/</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Mark Anthony Brown Jr.</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Strauch Early Career Fellow</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>mab692@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/mark-anthony-brown-jr/</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Matthew Connors</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Visiting Critic (summer 2026)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>imagetext@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>department_general</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/matthew-connors/</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Claire Donato</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Visiting Critic (summer and fall 2026)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Filmmaking</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>imagetext@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>department_general</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/claire-donato/</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Whitney Hubbs</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Visiting Critic (summer and fall 2026)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>weh62@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/whitney-hubbs/</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Kyle Bellucci Johanson</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Visiting Critic</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>kj368@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/kyle-bellucci-johanson/</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Ben Rivers</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Visiting Critic (summer 2026)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Filmmaking</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>imagetext@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>department_general</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/ben-rivers/</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Keisha Scarville</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Visiting Critic (fall 2026)</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>imagetext@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>department_general</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/keisha-scarville/</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Paulina Velázquez Solís</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Visiting Critic</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>pv233@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/paulina-velazquez-solis/</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Carla Williams</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Visiting Critic (summer 2026)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>imagetext@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>department_general</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/carla-williams/</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Cornell University, Department of Art (AAP)</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Carmen Winant</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Visiting Critic (summer 2026)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Art</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>cw297@cornell.edu</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>https://aap.cornell.edu/people/carmen-winant/</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A7:I35"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add faculty email scraping Batch 6: Syracuse, Slade (Tier 2 complete); UdK Berlin skipped
25 new faculty rows (Syracuse 4, Slade 21), bringing the master workbook to
16 schools and 531 total rows. Completes all attemptable Tier 2 schools -
UdK Berlin skipped after 3 URL attempts found no working staff directory
(first school this project has fully given up on for lack of a data
source, distinct from CIA which was scraped and confirmed to have none).

Both Syracuse and Slade needed a workaround from the brief's named URL:
Syracuse's real data lives on the /contact/ page (master directory is a
dead JS widget, confirmed independently); Slade's real academic roster is
at /people/academic/, not the /people/key-staff/ page the brief named
(which is admin/technical staff only).
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Faculty Scraping/master_faculty.xlsx
+++ b/Dezi Art Prize Faculty Scraping/master_faculty.xlsx
@@ -21,6 +21,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UIC" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rutgers" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cornell" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Syracuse" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slade" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Temple-Tyler'!$A$7:$I$58</definedName>
@@ -37,6 +39,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'UIC'!$A$7:$I$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Rutgers'!$A$7:$I$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Cornell'!$A$7:$I$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Syracuse'!$A$7:$I$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Slade'!$A$7:$I$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -6404,6 +6408,1397 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Country: United States</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>City: Syracuse, NY</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Source: Syracuse University, College of Visual and Performing Arts, School of Art - /academics/art/contact/ page (the master faculty-staff directory is a JS search widget with no default results, confirmed unusable per the brief). This page has the School of Art Director (medium classified from bio text on his own profile page - no discipline given on the contact page for this role) plus 4 'Area Leads' with a discipline label given directly (e.g. 'Printmaking', 'Illustration B.F.A.') but email only on their individual profile page. 1 area lead (Studio Arts B.F.A./B.S., generalist label with no specific medium) excluded rather than guessed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://vpa.syracuse.edu/academics/art/contact/ (plus 4 individual /faculty-staff/&lt;slug&gt;/ profile pages)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>school_name</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>faculty_name</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>email_type</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>date_extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Syracuse University, College of Visual and Performing Arts, School of Art</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Professor Robert Wysocki</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>School of Art Director</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>School of Art</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>rjwysock@syr.edu</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://vpa.syracuse.edu/academics/art/contact/</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Syracuse University, College of Visual and Performing Arts, School of Art</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Frank Cammuso</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Area Lead, Illustration B.F.A.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Illustration B.F.A.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>fvcammus@syr.edu</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://vpa.syracuse.edu/faculty-staff/cammuso-frank/</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Syracuse University, College of Visual and Performing Arts, School of Art</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Dusty Herbig</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Area Lead, Printmaking</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Printmaking</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Fiber and Material Arts</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>dtherbig@syr.edu</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://vpa.syracuse.edu/faculty-staff/herbig-dusty-1/</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Syracuse University, College of Visual and Performing Arts, School of Art</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Ekaterina Vanovskaya</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Area Lead, Drawing and Painting</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Drawing and Painting</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>evanovsk@syr.edu</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://vpa.syracuse.edu/faculty-staff/vanovskaya-ekaterina-1/</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A7:I11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Country: United Kingdom</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>City: London, England</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Source: Slade School of Fine Art, University College London (UCL) - /people/academic/ listing (46 people, single page, no pagination). Medium classified from title text shown directly on the listing (e.g. 'Lecturer, Painting', 'Associate Professor, Sculpture'); email only on individual profile pages - required a click-through pass for the 21 in-scope people.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://www.ucl.ac.uk/slade/people/academic/ (plus 21 individual profile pages)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>school_name</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>faculty_name</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>email_type</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>date_extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Kate Bright</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Associate Professor, Head of Undergraduate Sculpture (spring and summer terms 2024)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>k.bright@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/kbrig40/</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Peter Davies</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Lecturer, Painting</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>peter.davies@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/pdavi97/</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Jade de Montserrat</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Lecturer, Painting</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>j.montserrat@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/jdemo02/</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Lilah Fowler</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Associate Professor, Sculpture</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>l.fowler@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/lmfow09/</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Nadia Hebson</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Associate Professor, Co-Director of Studies, Graduate Programmes, Head of Graduate Painting, Graduate Tutor (MA/MFA)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>n.hebson@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/njheb06/</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Holly Hendry</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Lecturer, Sculpture</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>holly.hendry.09@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/hhend03/</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Neil Jeffries</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Lecturer, Painting</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>n.jeffries@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/nfjef05/</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Christine Kirubi</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Lecturer, Painting</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>christine.kirubi@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/cmkir12/</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Brighid Lowe</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Professor of Fine Art, Sculpture</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>b.lowe@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/blowe96/</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Onya McCausland</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Associate Professor, Head of Undergraduate Painting</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>o.mccausland@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/omcca29/</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Hayley Newman</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Associate Professor, Sculpture</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>h.newman@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/hjene78/</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Katrina Palmer</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Professor of Fine Art, Sculpture</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>katrina.palmer@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/kpalm97/</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Liz Rideal</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Professor of Fine Art, Painting</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>l.rideal@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/mecri22/</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Karin Ruggaber</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Professor of Fine Art, Head of Graduate Sculpture</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>k.ruggaber@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/krugg33/</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Adam Saad</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Lecturer, Painting</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>adam.saad@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/asaad11/</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Zeinab Saleh</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Lecturer, Painting</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>zeinab.saleh@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/zsale90/</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Gary Stevens</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Associate Professor, Sculpture</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>g.stevens@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/gstev52/</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Jack Strange</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Lecturer, Sculpture</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>jack.strange@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/jtdst45/</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Estelle Thompson</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Professor, Painting</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>estelle.thompson@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/ethom85/</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Phoebe Unwin</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Associate Professor, Painting</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>phoebe.unwin@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/pcunw18/</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Jo Volley</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Associate Professor, Painting</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>j.volley@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/jvoll94/</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A7:I28"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update master_faculty.xlsx with Batch 6 (Syracuse, Slade) - 531 total rows, Tier 2 complete
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Faculty Scraping/master_faculty.xlsx
+++ b/Dezi Art Prize Faculty Scraping/master_faculty.xlsx
@@ -21,6 +21,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UIC" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rutgers" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cornell" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Syracuse" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slade" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Temple-Tyler'!$A$7:$I$58</definedName>
@@ -37,6 +39,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'UIC'!$A$7:$I$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Rutgers'!$A$7:$I$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Cornell'!$A$7:$I$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Syracuse'!$A$7:$I$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Slade'!$A$7:$I$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -6404,6 +6408,1397 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Country: United States</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>City: Syracuse, NY</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Source: Syracuse University, College of Visual and Performing Arts, School of Art - /academics/art/contact/ page (the master faculty-staff directory is a JS search widget with no default results, confirmed unusable per the brief). This page has the School of Art Director (medium classified from bio text on his own profile page - no discipline given on the contact page for this role) plus 4 'Area Leads' with a discipline label given directly (e.g. 'Printmaking', 'Illustration B.F.A.') but email only on their individual profile page. 1 area lead (Studio Arts B.F.A./B.S., generalist label with no specific medium) excluded rather than guessed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://vpa.syracuse.edu/academics/art/contact/ (plus 4 individual /faculty-staff/&lt;slug&gt;/ profile pages)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>school_name</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>faculty_name</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>email_type</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>date_extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Syracuse University, College of Visual and Performing Arts, School of Art</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Professor Robert Wysocki</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>School of Art Director</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>School of Art</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>rjwysock@syr.edu</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>direct</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://vpa.syracuse.edu/academics/art/contact/</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Syracuse University, College of Visual and Performing Arts, School of Art</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Frank Cammuso</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Area Lead, Illustration B.F.A.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Illustration B.F.A.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>fvcammus@syr.edu</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://vpa.syracuse.edu/faculty-staff/cammuso-frank/</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Syracuse University, College of Visual and Performing Arts, School of Art</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Dusty Herbig</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Area Lead, Printmaking</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Printmaking</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Fiber and Material Arts</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>dtherbig@syr.edu</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://vpa.syracuse.edu/faculty-staff/herbig-dusty-1/</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Syracuse University, College of Visual and Performing Arts, School of Art</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Ekaterina Vanovskaya</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Area Lead, Drawing and Painting</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Drawing and Painting</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>evanovsk@syr.edu</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://vpa.syracuse.edu/faculty-staff/vanovskaya-ekaterina-1/</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A7:I11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Country: United Kingdom</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>City: London, England</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Source: Slade School of Fine Art, University College London (UCL) - /people/academic/ listing (46 people, single page, no pagination). Medium classified from title text shown directly on the listing (e.g. 'Lecturer, Painting', 'Associate Professor, Sculpture'); email only on individual profile pages - required a click-through pass for the 21 in-scope people.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://www.ucl.ac.uk/slade/people/academic/ (plus 21 individual profile pages)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>school_name</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>faculty_name</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>email_type</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>date_extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Kate Bright</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Associate Professor, Head of Undergraduate Sculpture (spring and summer terms 2024)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>k.bright@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/kbrig40/</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Peter Davies</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Lecturer, Painting</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>peter.davies@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/pdavi97/</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Jade de Montserrat</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Lecturer, Painting</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>j.montserrat@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/jdemo02/</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Lilah Fowler</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Associate Professor, Sculpture</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>l.fowler@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/lmfow09/</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Nadia Hebson</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Associate Professor, Co-Director of Studies, Graduate Programmes, Head of Graduate Painting, Graduate Tutor (MA/MFA)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>n.hebson@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/njheb06/</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Holly Hendry</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Lecturer, Sculpture</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>holly.hendry.09@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/hhend03/</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Neil Jeffries</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Lecturer, Painting</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>n.jeffries@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/nfjef05/</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Christine Kirubi</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Lecturer, Painting</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>christine.kirubi@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/cmkir12/</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Brighid Lowe</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Professor of Fine Art, Sculpture</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>b.lowe@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/blowe96/</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Onya McCausland</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Associate Professor, Head of Undergraduate Painting</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>o.mccausland@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/omcca29/</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Hayley Newman</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Associate Professor, Sculpture</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>h.newman@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/hjene78/</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Katrina Palmer</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Professor of Fine Art, Sculpture</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>katrina.palmer@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/kpalm97/</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Liz Rideal</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Professor of Fine Art, Painting</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>l.rideal@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/mecri22/</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Karin Ruggaber</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Professor of Fine Art, Head of Graduate Sculpture</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>k.ruggaber@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/krugg33/</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Adam Saad</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Lecturer, Painting</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>adam.saad@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/asaad11/</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Zeinab Saleh</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Lecturer, Painting</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>zeinab.saleh@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/zsale90/</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Gary Stevens</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Associate Professor, Sculpture</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>g.stevens@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/gstev52/</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Jack Strange</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Lecturer, Sculpture</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>jack.strange@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/jtdst45/</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Estelle Thompson</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Professor, Painting</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>estelle.thompson@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/ethom85/</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Phoebe Unwin</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Associate Professor, Painting</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>phoebe.unwin@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/pcunw18/</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art, University College London (UCL)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Jo Volley</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Associate Professor, Painting</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Slade School of Fine Art</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>j.volley@ucl.ac.uk</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://www.ucl.ac.uk/slade/people/academic/jvoll94/</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A7:I28"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add faculty email scraping Batch 7: Yale, CMU, GSA, Kunstakademie Dusseldorf
50 new faculty rows found by re-checking Tier 3 schools the brief said had
no individual emails - Yale (6), CMU (14), GSA (29), and Kunstakademie
Dusseldorf (1) all had real emails on individual profile pages that the
brief's page-level check missed. Bringing the master workbook to 20
schools and 611 total rows.

Also caught and reversed a fabricated WebFetch response for Gerrit
Rietveld Academie (invented department-head names/emails that don't
exist on the real page, confirmed via direct fetch) before it was
committed - logged in ISSUES_LOG.md as a process note.
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Faculty Scraping/master_faculty.xlsx
+++ b/Dezi Art Prize Faculty Scraping/master_faculty.xlsx
@@ -23,6 +23,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cornell" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Syracuse" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slade" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yale" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CMU" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GSA" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kunstakademie Dusseldorf" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Temple-Tyler'!$A$7:$I$58</definedName>
@@ -41,6 +45,10 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Cornell'!$A$7:$I$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Syracuse'!$A$7:$I$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Slade'!$A$7:$I$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Yale'!$A$7:$I$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'CMU'!$A$7:$I$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'GSA'!$A$7:$I$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'Kunstakademie Dusseldorf'!$A$7:$I$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -7799,6 +7807,2509 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Country: United States</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>City: New Haven, CT</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Source: Yale School of Art - the brief correctly found the /about/people/faculty-and-staff listing page has no emails, classifying Yale as Tier 3. However each of the 74 people listed (Academic Leadership, Graphic Design, Painting/Printmaking, Photography, Sculpture, Interdepartmental, Undergraduate, Yale Norfolk, Faculty Emeriti sections; Faculty Governing Board and Administration/Staff excluded) links to their own profile page, and SOME publish a direct email there (appears to be individual choice - several senior faculty link to a personal site/Substack instead). Only 6 of 49 in-scope profiles checked had a public email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://www.art.yale.edu/about/people/faculty-and-staff (plus 49 individual /&lt;Name&gt; profile pages)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>school_name</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>faculty_name</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>email_type</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>date_extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Yale School of Art</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Anoka Faruqee</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Associate Dean; Professor in Painting/Printmaking</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>academic leadership</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>anoka.faruqee@yale.edu</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://www.art.yale.edu/AnokaFaruqee</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Yale School of Art</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Yeju Choi</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Senior Critic</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>graphic design</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>yeju.choi@yale.edu</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://www.art.yale.edu/YejuChoi</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Yale School of Art</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Anahita Vossoughi</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Critic; Associate Director of Digital Media</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>painting / printmaking</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>anahita.vossoughi@yale.edu</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://www.art.yale.edu/AnahitaVossoughi</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Yale School of Art</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Sam Contis</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Senior Critic</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>photography</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>sam.contis@yale.edu</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://www.art.yale.edu/SamContis</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Yale School of Art</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Matthew Leifheit</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Critic</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>photography</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>leifheit.matthew@gmail.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://www.art.yale.edu/MatthewLeifheit</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Yale School of Art</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Eva O'Leary</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Critic</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>photography</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>eva.oleary@yale.edu</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://www.art.yale.edu/EvaOLeary</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A7:I13"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Country: United States</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>City: Pittsburgh, PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Source: Carnegie Mellon University, School of Art - the brief's warning ("directory requires Andrew login, do NOT scrape") correctly applies to CMU's university-wide people directory, which was NOT used here. This is a different, fully public page - art.cmu.edu/people/faculty/ - the School of Art's own faculty listing, not login-walled. Individual profile pages publish a real institutional email (@andrew.cmu.edu or @cmu.edu) in a structured JSON metadata field. Medium classified from the discipline label shown directly on the listing (e.g. 'Drawing, Painting, Print, &amp; Photo', 'Electronic &amp; Time Based Media' - the latter mapped to Filmmaking as the closest of the 9 in-scope mediums, though it also covers interactive/digital work; an approximate call).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://art.cmu.edu/people/faculty/ (plus 14 individual /people/&lt;slug&gt;/ pages)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>school_name</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>faculty_name</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>email_type</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>date_extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Kim Beck</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Professor of Art</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Drawing, Painting, Print, &amp; Photo</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>kimbeck@andrew.cmu.edu</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/kim-beck/</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Meghana Bisineer</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Electronic &amp; Time Based Media</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Filmmaking</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>mbisinee@andrew.cmu.edu</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/meghana-bisineer/</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Johannes DeYoung</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Associate Professor of Art</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Electronic &amp; Time Based Media</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Filmmaking</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>jsdeyoung@cmu.edu</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/johannes-deyoung/</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Isla Hansen</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Art</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Sculpture, Installation, &amp; Site Work</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>ihansen@andrew.cmu.edu</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/isla-hansen/</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Sujin Kim</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Associate Professor of Art</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Electronic &amp; Time Based Media</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Filmmaking</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>kimsujin@cmu.edu</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/sujin-kim/</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Golan Levin</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Professor of Art</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Electronic &amp; Time Based Media</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Filmmaking</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>golan@andrew.cmu.edu</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/golan-levin/</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Clayton Merrell</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Dorothy L. Stubnitz Professor of Art</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Drawing, Painting, Print, &amp; Photo</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>cmerrell@andrew.cmu.edu</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/clayton-merrell/</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Paolo Pedercini</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Associate Professor of Art</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Electronic &amp; Time Based Media</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Filmmaking</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>paolop@cmu.edu</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/paolo-pedercini/</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Rich Pell</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Associate Professor of Art</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Electronic &amp; Time Based Media</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Filmmaking</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>rp3h@andrew.cmu.edu</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/rich-pell/</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Britt Ransom</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Associate Professor of Art</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Sculpture, Installation, &amp; Site Work</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>brittanr@andrew.cmu.edu</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/britt-ransom/</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Sharmistha Ray</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Estella Loomis McCandless Assistant Professor of Art</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Drawing, Painting, Print, &amp; Photo</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>sharmisr@andrew.cmu.edu</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/sharmistha-ray/</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Yoko Sekino-Bové</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Assistant Teaching Professor of Art</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Sculpture, Installation, &amp; Site Work</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>ysekinob@andrew.cmu.edu</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/yoko-sekino-bove/</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Jamie Wolfe</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Art</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Electronic &amp; Time Based Media</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Filmmaking</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>jamiewol@andrew.cmu.edu</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/jamie-wolfe/</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Imin Yeh</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Drawing, Painting, Print, &amp; Photo</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>iminyeh@cmu.edu</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/imin-yeh/</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A7:I21"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Country: United Kingdom</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>City: Glasgow, Scotland</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Source: Glasgow School of Art - the brief correctly found the /staff listing page has no emails, classifying GSA as Tier 3. However individual profile pages DO publish a real email (e.g. 'Email: N.Oddy@gsa.ac.uk') even though the listing itself doesn't show it. ~197 total staff across all departments (architecture, design history, admin, etc., 2 pages); medium classified from job title text, keeping only the ~29 whose title names an in-scope medium (e.g. 'Lecturer in Painting and Printmaking', 'Lecturer Sculpture and Environmental Art').</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://www.gsa.ac.uk/staff (2 pages, plus ~29 individual /staff/user-&lt;id&gt; pages)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>school_name</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>faculty_name</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>email_type</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>date_extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Aoife McGarrigle</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Pathway Tutor M.Litt Print Media, Lithography technician, Team Leader TSD Print</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Fiber and Material Arts</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>A.McGarrigle@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-230</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Annette Heyer</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Lecturer in Painting and Printmaking</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>A.Heyer@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-231</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Justin Carter</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Lecturer in Sculpture &amp; Environmental Art</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>J.Carter@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-239</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Peter McCaughey</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Lecturer Sculpture and Environmental Art</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>P.McCaughey@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-240</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Christina McBride</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Lecturer Master of Fine Art (MFA) and Fine Art Photography</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>C.McBride@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-253</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Lesley Punton</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Head of Fine Art Photography</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>L.Punton@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-281</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Anna Gordon</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>head of department and programme leader, silversmithing and jewellery</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>A.Gordon@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-284</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Ronan Breslin</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Lecturer Sound for the Moving Image</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Filmmaking</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>R.Breslin@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-316</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Eddie Stewart</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Lecturer Painting &amp; Printmaking</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Ed.Stewart@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-395</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Stephanie Smith</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Lecturer Sculpture Environmental Art / PhD Primary &amp; Secondary Supervisor</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>S.Smith@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-401</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Dr Graham Lister</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Lecturer - Painting and Printmaking</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>G.Lister@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-412</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Michael Mersinis</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Lecturer in Fine Art Photography</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>M.Mersinis@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-448</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Chris Wallace</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>P/T Lecturer Product Design Engineering</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>C.Wallace@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-656</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Paul Maguire</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Programme Leader, BA (Hons) Interaction Design</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>UI/UX Design</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>P.Maguire@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-722</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Kirsty Ross</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Lecturer and Final Year Coordinator, Department of Product Design, the Innovation School</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>K.Ross@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-754</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Fiona Ann Jardine</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Programme Leader, Fashion Narrative</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Fashion</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>F.Jardine@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-925</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Dr Michael Stubbs</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Reader in Contemporary Painting</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>M.Stubbs@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-1024</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Chris Hand</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Lecturer and subject lead for Interaction Design</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>UI/UX Design</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>C.Hand@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-1061</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Jessica Argo</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Programme Leader, BDes Sound for Moving Image</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Filmmaking</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>J.Argo@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-1072</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Marianne Anderson</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Lecturer, Silversmithing &amp; Jewellery</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>M.Anderson@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-1162</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Becky Šik</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Lecturer in Sculpture and Environmental Art</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>B.Sik@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-1271</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Anne-Marie Copestake</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Lecturer Fine Art Photography</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>A.Copestake@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-1420</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Sara Barker</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Head of Sculpture and Environmental Art</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>S.Barker@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-1469</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Dr Zoe Mendelson</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Head of Painting &amp; Printmaking</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>z.mendelson@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-1584</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Marita Fraser</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>UG Programme Director and Interim Head of Sculpture and Environmental Art,</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>m.fraser@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-1613</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Owain McGilvary</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Lecturer in Painting &amp; Printmaking</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>O.McGilvary@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-1658</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Rachel Adams</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Lecturer in Sculpture and Environmental Art</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>R.Adams@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-1679</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Karen David</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Lecturer in Painting &amp; Printmaking</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>k.david@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-1686</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Matthew Williams</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Photography Lecturer</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>m.williams@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-1848</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A7:I36"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -10343,6 +12854,161 @@
     </row>
   </sheetData>
   <autoFilter ref="A7:I59"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Country: Germany</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>City: Dusseldorf</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Source: Kunstakademie Dusseldorf - the brief's Tier 3 classification (no emails, use postmaster@) is correct for the vast majority: checked all 24 'Freie Kunst' (Free Art) professors' individual profile pages (JS-rendered, required crawl4ai) and only 1 (Alexandra Bircken) publishes an email, included in her application-instructions text ('send your portfolio to alexandra.bircken@kunstakademie-duesseldorf.de'). The other 23 genuinely have no email anywhere on their page, confirmed by direct inspection, not a fetch failure. Baukunst (Architecture) and Kunstbezogene Wissenschaften (art theory/sciences) sections excluded as out of scope.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://kunstakademie-duesseldorf.de/studienangebot-und-bewerbung/professor-innen/ (plus 24 individual profile pages)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>school_name</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>faculty_name</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>email_type</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>date_extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Kunstakademie Dusseldorf (Dusseldorf Art Academy)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Prof.in Alexandra Bircken</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Professor, Freie Kunst</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Freie Kunst</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>alexandra.bircken@kunstakademie-duesseldorf.de</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://kunstakademie-duesseldorf.de/studienangebot-und-bewerbung/professor-innen/prof-in-alexandra-bircken/</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A7:I8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update master_faculty.xlsx with Batch 7 (Yale, CMU, GSA, Dusseldorf) - 611 total rows
</commit_message>
<xml_diff>
--- a/Dezi Art Prize Faculty Scraping/master_faculty.xlsx
+++ b/Dezi Art Prize Faculty Scraping/master_faculty.xlsx
@@ -23,6 +23,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cornell" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Syracuse" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slade" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yale" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CMU" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GSA" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kunstakademie Dusseldorf" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Temple-Tyler'!$A$7:$I$58</definedName>
@@ -41,6 +45,10 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Cornell'!$A$7:$I$35</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Syracuse'!$A$7:$I$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Slade'!$A$7:$I$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Yale'!$A$7:$I$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'CMU'!$A$7:$I$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'GSA'!$A$7:$I$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'Kunstakademie Dusseldorf'!$A$7:$I$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -7799,6 +7807,2509 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Country: United States</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>City: New Haven, CT</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Source: Yale School of Art - the brief correctly found the /about/people/faculty-and-staff listing page has no emails, classifying Yale as Tier 3. However each of the 74 people listed (Academic Leadership, Graphic Design, Painting/Printmaking, Photography, Sculpture, Interdepartmental, Undergraduate, Yale Norfolk, Faculty Emeriti sections; Faculty Governing Board and Administration/Staff excluded) links to their own profile page, and SOME publish a direct email there (appears to be individual choice - several senior faculty link to a personal site/Substack instead). Only 6 of 49 in-scope profiles checked had a public email.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://www.art.yale.edu/about/people/faculty-and-staff (plus 49 individual /&lt;Name&gt; profile pages)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>school_name</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>faculty_name</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>email_type</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>date_extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Yale School of Art</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Anoka Faruqee</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Associate Dean; Professor in Painting/Printmaking</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>academic leadership</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>anoka.faruqee@yale.edu</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://www.art.yale.edu/AnokaFaruqee</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Yale School of Art</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Yeju Choi</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Senior Critic</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>graphic design</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>yeju.choi@yale.edu</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://www.art.yale.edu/YejuChoi</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Yale School of Art</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Anahita Vossoughi</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Critic; Associate Director of Digital Media</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>painting / printmaking</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>anahita.vossoughi@yale.edu</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://www.art.yale.edu/AnahitaVossoughi</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Yale School of Art</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Sam Contis</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Senior Critic</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>photography</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>sam.contis@yale.edu</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://www.art.yale.edu/SamContis</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Yale School of Art</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Matthew Leifheit</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Critic</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>photography</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>leifheit.matthew@gmail.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://www.art.yale.edu/MatthewLeifheit</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Yale School of Art</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Eva O'Leary</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Critic</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>photography</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>eva.oleary@yale.edu</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://www.art.yale.edu/EvaOLeary</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A7:I13"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Country: United States</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>City: Pittsburgh, PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Source: Carnegie Mellon University, School of Art - the brief's warning ("directory requires Andrew login, do NOT scrape") correctly applies to CMU's university-wide people directory, which was NOT used here. This is a different, fully public page - art.cmu.edu/people/faculty/ - the School of Art's own faculty listing, not login-walled. Individual profile pages publish a real institutional email (@andrew.cmu.edu or @cmu.edu) in a structured JSON metadata field. Medium classified from the discipline label shown directly on the listing (e.g. 'Drawing, Painting, Print, &amp; Photo', 'Electronic &amp; Time Based Media' - the latter mapped to Filmmaking as the closest of the 9 in-scope mediums, though it also covers interactive/digital work; an approximate call).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://art.cmu.edu/people/faculty/ (plus 14 individual /people/&lt;slug&gt;/ pages)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>school_name</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>faculty_name</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>email_type</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>date_extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Kim Beck</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Professor of Art</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Drawing, Painting, Print, &amp; Photo</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>kimbeck@andrew.cmu.edu</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/kim-beck/</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Meghana Bisineer</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Electronic &amp; Time Based Media</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Filmmaking</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>mbisinee@andrew.cmu.edu</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/meghana-bisineer/</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Johannes DeYoung</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Associate Professor of Art</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Electronic &amp; Time Based Media</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Filmmaking</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>jsdeyoung@cmu.edu</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/johannes-deyoung/</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Isla Hansen</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Art</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Sculpture, Installation, &amp; Site Work</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>ihansen@andrew.cmu.edu</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/isla-hansen/</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Sujin Kim</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Associate Professor of Art</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Electronic &amp; Time Based Media</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Filmmaking</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>kimsujin@cmu.edu</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/sujin-kim/</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Golan Levin</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Professor of Art</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Electronic &amp; Time Based Media</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Filmmaking</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>golan@andrew.cmu.edu</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/golan-levin/</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Clayton Merrell</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Dorothy L. Stubnitz Professor of Art</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Drawing, Painting, Print, &amp; Photo</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>cmerrell@andrew.cmu.edu</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/clayton-merrell/</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Paolo Pedercini</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Associate Professor of Art</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Electronic &amp; Time Based Media</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Filmmaking</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>paolop@cmu.edu</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/paolo-pedercini/</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Rich Pell</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Associate Professor of Art</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Electronic &amp; Time Based Media</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Filmmaking</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>rp3h@andrew.cmu.edu</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/rich-pell/</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Britt Ransom</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Associate Professor of Art</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Sculpture, Installation, &amp; Site Work</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>brittanr@andrew.cmu.edu</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/britt-ransom/</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Sharmistha Ray</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Estella Loomis McCandless Assistant Professor of Art</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Drawing, Painting, Print, &amp; Photo</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>sharmisr@andrew.cmu.edu</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/sharmistha-ray/</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Yoko Sekino-Bové</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Assistant Teaching Professor of Art</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Sculpture, Installation, &amp; Site Work</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>ysekinob@andrew.cmu.edu</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/yoko-sekino-bove/</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Jamie Wolfe</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Assistant Professor of Art</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Electronic &amp; Time Based Media</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Filmmaking</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>jamiewol@andrew.cmu.edu</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/jamie-wolfe/</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University, School of Art</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Imin Yeh</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Drawing, Painting, Print, &amp; Photo</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>iminyeh@cmu.edu</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://art.cmu.edu/people/imin-yeh/</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A7:I21"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Country: United Kingdom</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>City: Glasgow, Scotland</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Source: Glasgow School of Art - the brief correctly found the /staff listing page has no emails, classifying GSA as Tier 3. However individual profile pages DO publish a real email (e.g. 'Email: N.Oddy@gsa.ac.uk') even though the listing itself doesn't show it. ~197 total staff across all departments (architecture, design history, admin, etc., 2 pages); medium classified from job title text, keeping only the ~29 whose title names an in-scope medium (e.g. 'Lecturer in Painting and Printmaking', 'Lecturer Sculpture and Environmental Art').</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://www.gsa.ac.uk/staff (2 pages, plus ~29 individual /staff/user-&lt;id&gt; pages)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>school_name</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>faculty_name</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>email_type</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>date_extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Aoife McGarrigle</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Pathway Tutor M.Litt Print Media, Lithography technician, Team Leader TSD Print</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Fiber and Material Arts</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>A.McGarrigle@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-230</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Annette Heyer</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Lecturer in Painting and Printmaking</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>A.Heyer@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-231</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Justin Carter</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Lecturer in Sculpture &amp; Environmental Art</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>J.Carter@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-239</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Peter McCaughey</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Lecturer Sculpture and Environmental Art</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>P.McCaughey@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-240</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Christina McBride</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Lecturer Master of Fine Art (MFA) and Fine Art Photography</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>C.McBride@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-253</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Lesley Punton</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Head of Fine Art Photography</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>L.Punton@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-281</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Anna Gordon</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>head of department and programme leader, silversmithing and jewellery</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>A.Gordon@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-284</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Ronan Breslin</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Lecturer Sound for the Moving Image</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Filmmaking</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>R.Breslin@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-316</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Eddie Stewart</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Lecturer Painting &amp; Printmaking</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Ed.Stewart@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-395</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Stephanie Smith</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Lecturer Sculpture Environmental Art / PhD Primary &amp; Secondary Supervisor</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>S.Smith@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-401</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Dr Graham Lister</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Lecturer - Painting and Printmaking</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>G.Lister@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-412</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Michael Mersinis</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Lecturer in Fine Art Photography</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>M.Mersinis@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-448</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Chris Wallace</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>P/T Lecturer Product Design Engineering</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>C.Wallace@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-656</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Paul Maguire</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Programme Leader, BA (Hons) Interaction Design</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>UI/UX Design</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>P.Maguire@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-722</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Kirsty Ross</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Lecturer and Final Year Coordinator, Department of Product Design, the Innovation School</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>K.Ross@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-754</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Fiona Ann Jardine</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Programme Leader, Fashion Narrative</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Fashion</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>F.Jardine@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-925</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Dr Michael Stubbs</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Reader in Contemporary Painting</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>M.Stubbs@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-1024</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Chris Hand</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Lecturer and subject lead for Interaction Design</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>UI/UX Design</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>C.Hand@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-1061</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Jessica Argo</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Programme Leader, BDes Sound for Moving Image</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Filmmaking</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>J.Argo@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-1072</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Marianne Anderson</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Lecturer, Silversmithing &amp; Jewellery</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>M.Anderson@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-1162</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Becky Šik</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Lecturer in Sculpture and Environmental Art</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>B.Sik@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-1271</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Anne-Marie Copestake</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Lecturer Fine Art Photography</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>A.Copestake@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-1420</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Sara Barker</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Head of Sculpture and Environmental Art</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>S.Barker@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-1469</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Dr Zoe Mendelson</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Head of Painting &amp; Printmaking</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>z.mendelson@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-1584</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Marita Fraser</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>UG Programme Director and Interim Head of Sculpture and Environmental Art,</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>m.fraser@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-1613</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Owain McGilvary</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Lecturer in Painting &amp; Printmaking</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>O.McGilvary@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-1658</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Rachel Adams</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Lecturer in Sculpture and Environmental Art</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>R.Adams@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-1679</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Karen David</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Lecturer in Painting &amp; Printmaking</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Painting/Drawing</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>k.david@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-1686</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Glasgow School of Art</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Matthew Williams</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Photography Lecturer</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Photography</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>m.williams@gsa.ac.uk</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>https://www.gsa.ac.uk/staff/user-1848</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A7:I36"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -10343,6 +12854,161 @@
     </row>
   </sheetData>
   <autoFilter ref="A7:I59"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Country: Germany</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>City: Dusseldorf</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Source: Kunstakademie Dusseldorf - the brief's Tier 3 classification (no emails, use postmaster@) is correct for the vast majority: checked all 24 'Freie Kunst' (Free Art) professors' individual profile pages (JS-rendered, required crawl4ai) and only 1 (Alexandra Bircken) publishes an email, included in her application-instructions text ('send your portfolio to alexandra.bircken@kunstakademie-duesseldorf.de'). The other 23 genuinely have no email anywhere on their page, confirmed by direct inspection, not a fetch failure. Baukunst (Architecture) and Kunstbezogene Wissenschaften (art theory/sciences) sections excluded as out of scope.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>URL: https://kunstakademie-duesseldorf.de/studienangebot-und-bewerbung/professor-innen/ (plus 24 individual profile pages)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Accessed: 2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>school_name</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>faculty_name</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>department</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>email_type</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>date_extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Kunstakademie Dusseldorf (Dusseldorf Art Academy)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Prof.in Alexandra Bircken</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Professor, Freie Kunst</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Freie Kunst</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Sculpture</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>alexandra.bircken@kunstakademie-duesseldorf.de</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://kunstakademie-duesseldorf.de/studienangebot-und-bewerbung/professor-innen/prof-in-alexandra-bircken/</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A7:I8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>